<commit_message>
FSL Plaus commit 07022025
Updates to correct penalty scores displayed in the html output.

This impacted the following files:
- resources/overall_plaus.xlsx
- calculate_plausibility.R

On a secondary note, made a minor change to include add_fcs and a recoding for dnk and pnta values in the HHS indicator, which were erroneously allowed in the MSNA template tool this year. Proper FCS, HHS, rCSI and LCSI variables are needed for the report to calculate plausibility, so these functions are needed if the dataset doesnt already have proper formatting.
</commit_message>
<xml_diff>
--- a/inst/fsl_quality_report/resources/overall_plaus.xlsx
+++ b/inst/fsl_quality_report/resources/overall_plaus.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\impactR4PHU\inst\fsl_quality_report\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted-my.sharepoint.com/personal/saeed_rahman_impact-initiatives_org/Documents/R Projects/impactR4PHU/inst/fsl_quality_report/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2708F7E-EB57-4B3E-B12E-2672C83A8B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{D2708F7E-EB57-4B3E-B12E-2672C83A8B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37EE582D-5E48-4C0A-8B31-09E75583990F}"/>
   <bookViews>
-    <workbookView xWindow="5790" yWindow="3060" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16200" windowWidth="12840" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FSL" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="102">
   <si>
     <t>flag_name</t>
   </si>
@@ -55,9 +55,6 @@
     <t xml:space="preserve">Problematic </t>
   </si>
   <si>
-    <t>&lt;2%</t>
-  </si>
-  <si>
     <t>&gt;10%</t>
   </si>
   <si>
@@ -173,9 +170,6 @@
   </si>
   <si>
     <t>plaus_fsl_cat</t>
-  </si>
-  <si>
-    <t>2-&lt;10%</t>
   </si>
   <si>
     <t>plaus_ageratio</t>
@@ -803,96 +797,102 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -902,25 +902,19 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1225,588 +1219,588 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
     </row>
     <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="23"/>
+      <c r="D2" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="25"/>
+      <c r="F2" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="26"/>
+    </row>
+    <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="43"/>
+      <c r="B3" s="41">
+        <v>0</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="41">
+        <v>2</v>
+      </c>
+      <c r="E3" s="42"/>
+      <c r="F3" s="47">
+        <v>4</v>
+      </c>
+      <c r="G3" s="47"/>
+    </row>
+    <row r="4" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="38"/>
+      <c r="D4" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="38"/>
+      <c r="F4" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="32"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="36"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+    </row>
+    <row r="6" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="36"/>
+      <c r="B6" s="41">
+        <v>0</v>
+      </c>
+      <c r="C6" s="42"/>
+      <c r="D6" s="29">
+        <v>1</v>
+      </c>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29">
+        <v>2</v>
+      </c>
+      <c r="G6" s="29"/>
+    </row>
+    <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="25"/>
+      <c r="F7" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="26"/>
+    </row>
+    <row r="8" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="43"/>
+      <c r="B8" s="27">
+        <v>0</v>
+      </c>
+      <c r="C8" s="28"/>
+      <c r="D8" s="27">
+        <v>1</v>
+      </c>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29">
+        <v>2</v>
+      </c>
+      <c r="G8" s="29"/>
+    </row>
+    <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="23"/>
+      <c r="D9" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="25"/>
+      <c r="F9" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="26"/>
+    </row>
+    <row r="10" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="43"/>
+      <c r="B10" s="27">
+        <v>0</v>
+      </c>
+      <c r="C10" s="28"/>
+      <c r="D10" s="27">
+        <v>2</v>
+      </c>
+      <c r="E10" s="28"/>
+      <c r="F10" s="29">
+        <v>4</v>
+      </c>
+      <c r="G10" s="29"/>
+    </row>
+    <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B11" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="23"/>
+      <c r="D11" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="26"/>
+    </row>
+    <row r="12" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="43"/>
+      <c r="B12" s="27">
+        <v>0</v>
+      </c>
+      <c r="C12" s="28"/>
+      <c r="D12" s="27">
+        <v>1</v>
+      </c>
+      <c r="E12" s="28"/>
+      <c r="F12" s="29">
+        <v>2</v>
+      </c>
+      <c r="G12" s="29"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="23"/>
+      <c r="D13" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="25"/>
+      <c r="F13" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="26"/>
+    </row>
+    <row r="14" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="31"/>
+      <c r="B14" s="27">
+        <v>0</v>
+      </c>
+      <c r="C14" s="28"/>
+      <c r="D14" s="27">
+        <v>2</v>
+      </c>
+      <c r="E14" s="28"/>
+      <c r="F14" s="29">
+        <v>4</v>
+      </c>
+      <c r="G14" s="29"/>
+    </row>
+    <row r="15" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="23"/>
+      <c r="D15" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15" s="25"/>
+      <c r="F15" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="26"/>
+    </row>
+    <row r="16" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="30"/>
+      <c r="B16" s="33">
+        <v>0</v>
+      </c>
+      <c r="C16" s="34"/>
+      <c r="D16" s="33">
+        <v>2</v>
+      </c>
+      <c r="E16" s="34"/>
+      <c r="F16" s="44">
+        <v>4</v>
+      </c>
+      <c r="G16" s="44"/>
+    </row>
+    <row r="17" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="23"/>
+      <c r="D17" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="25"/>
+      <c r="F17" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" s="26"/>
+    </row>
+    <row r="18" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="43"/>
+      <c r="B18" s="27">
+        <v>0</v>
+      </c>
+      <c r="C18" s="28"/>
+      <c r="D18" s="27">
+        <v>4</v>
+      </c>
+      <c r="E18" s="28"/>
+      <c r="F18" s="29">
+        <v>6</v>
+      </c>
+      <c r="G18" s="29"/>
+    </row>
+    <row r="19" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="38"/>
+      <c r="D19" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="38"/>
+      <c r="F19" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="32"/>
+    </row>
+    <row r="20" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="36"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+    </row>
+    <row r="21" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="36"/>
+      <c r="B21" s="27">
+        <v>0</v>
+      </c>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29">
+        <v>2</v>
+      </c>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29">
+        <v>3</v>
+      </c>
+      <c r="G21" s="29"/>
+    </row>
+    <row r="22" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="50"/>
+      <c r="D22" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="25"/>
+      <c r="F22" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="51"/>
+    </row>
+    <row r="23" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="48"/>
+      <c r="B23" s="27">
+        <v>0</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="27">
+        <v>4</v>
+      </c>
+      <c r="E23" s="28"/>
+      <c r="F23" s="29">
+        <v>5</v>
+      </c>
+      <c r="G23" s="29"/>
+    </row>
+    <row r="24" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="23"/>
+      <c r="D24" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="25"/>
+      <c r="F24" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" s="26"/>
+    </row>
+    <row r="25" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="30"/>
+      <c r="B25" s="33">
+        <v>0</v>
+      </c>
+      <c r="C25" s="34"/>
+      <c r="D25" s="33">
+        <v>2</v>
+      </c>
+      <c r="E25" s="34"/>
+      <c r="F25" s="44">
+        <v>3</v>
+      </c>
+      <c r="G25" s="44"/>
+    </row>
+    <row r="26" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="55"/>
+      <c r="D26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E2" s="23"/>
-      <c r="F2" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="44"/>
-    </row>
-    <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="28"/>
-      <c r="B3" s="45">
-        <v>0</v>
-      </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="45">
-        <v>2</v>
-      </c>
-      <c r="E3" s="46"/>
-      <c r="F3" s="40">
-        <v>4</v>
-      </c>
-      <c r="G3" s="40"/>
-    </row>
-    <row r="4" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="56" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="56" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="57"/>
-      <c r="F4" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="30"/>
-    </row>
-    <row r="5" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
-      <c r="B5" s="58"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-    </row>
-    <row r="6" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="39"/>
-      <c r="B6" s="45">
-        <v>0</v>
-      </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="38">
-        <v>1</v>
-      </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38">
-        <v>2</v>
-      </c>
-      <c r="G6" s="38"/>
-    </row>
-    <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E7" s="23"/>
-      <c r="F7" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="44"/>
-    </row>
-    <row r="8" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="28"/>
-      <c r="B8" s="26">
-        <v>0</v>
-      </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="26">
-        <v>1</v>
-      </c>
-      <c r="E8" s="27"/>
-      <c r="F8" s="38">
-        <v>2</v>
-      </c>
-      <c r="G8" s="38"/>
-    </row>
-    <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="43"/>
-      <c r="D9" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G9" s="44"/>
-    </row>
-    <row r="10" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="28"/>
-      <c r="B10" s="26">
-        <v>0</v>
-      </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="26">
-        <v>2</v>
-      </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="38">
-        <v>4</v>
-      </c>
-      <c r="G10" s="38"/>
-    </row>
-    <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="43"/>
-      <c r="D11" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="44"/>
-    </row>
-    <row r="12" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-      <c r="B12" s="26">
-        <v>0</v>
-      </c>
-      <c r="C12" s="27"/>
-      <c r="D12" s="26">
-        <v>1</v>
-      </c>
-      <c r="E12" s="27"/>
-      <c r="F12" s="38">
-        <v>2</v>
-      </c>
-      <c r="G12" s="38"/>
-    </row>
-    <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="50" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E13" s="23"/>
-      <c r="F13" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="44"/>
-    </row>
-    <row r="14" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="61"/>
-      <c r="B14" s="26">
-        <v>0</v>
-      </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="26">
-        <v>2</v>
-      </c>
-      <c r="E14" s="27"/>
-      <c r="F14" s="38">
-        <v>4</v>
-      </c>
-      <c r="G14" s="38"/>
-    </row>
-    <row r="15" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="43"/>
-      <c r="D15" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G15" s="44"/>
-    </row>
-    <row r="16" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="50"/>
-      <c r="B16" s="24">
-        <v>0</v>
-      </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="24">
-        <v>2</v>
-      </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="51">
-        <v>4</v>
-      </c>
-      <c r="G16" s="51"/>
-    </row>
-    <row r="17" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="43"/>
-      <c r="D17" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E17" s="23"/>
-      <c r="F17" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" s="44"/>
-    </row>
-    <row r="18" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
-      <c r="B18" s="26">
-        <v>0</v>
-      </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="26">
-        <v>4</v>
-      </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="38">
-        <v>6</v>
-      </c>
-      <c r="G18" s="38"/>
-    </row>
-    <row r="19" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="56" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="57"/>
-      <c r="D19" s="56" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="57"/>
-      <c r="F19" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="30"/>
-    </row>
-    <row r="20" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
-      <c r="B20" s="58"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-    </row>
-    <row r="21" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
-      <c r="B21" s="26">
-        <v>0</v>
-      </c>
-      <c r="C21" s="27"/>
-      <c r="D21" s="38">
-        <v>2</v>
-      </c>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38">
-        <v>3</v>
-      </c>
-      <c r="G21" s="38"/>
-    </row>
-    <row r="22" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="55" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="36"/>
-      <c r="D22" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E22" s="23"/>
-      <c r="F22" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="G22" s="37"/>
-    </row>
-    <row r="23" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="55"/>
-      <c r="B23" s="26">
-        <v>0</v>
-      </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="26">
-        <v>4</v>
-      </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="38">
-        <v>5</v>
-      </c>
-      <c r="G23" s="38"/>
-    </row>
-    <row r="24" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E24" s="23"/>
-      <c r="F24" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G24" s="44"/>
-    </row>
-    <row r="25" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="50"/>
-      <c r="B25" s="24">
-        <v>0</v>
-      </c>
-      <c r="C25" s="25"/>
-      <c r="D25" s="24">
-        <v>2</v>
-      </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="51">
-        <v>3</v>
-      </c>
-      <c r="G25" s="51"/>
-    </row>
-    <row r="26" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="53"/>
-      <c r="D26" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="F26" s="54" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" s="54"/>
+      <c r="G26" s="56"/>
     </row>
     <row r="27" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28"/>
-      <c r="B27" s="26">
-        <v>0</v>
-      </c>
-      <c r="C27" s="27"/>
+      <c r="A27" s="43"/>
+      <c r="B27" s="27">
+        <v>0</v>
+      </c>
+      <c r="C27" s="28"/>
       <c r="D27" s="2">
         <v>6</v>
       </c>
       <c r="E27" s="2">
         <v>8</v>
       </c>
-      <c r="F27" s="38">
+      <c r="F27" s="29">
         <v>10</v>
       </c>
-      <c r="G27" s="38"/>
+      <c r="G27" s="29"/>
     </row>
     <row r="28" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="49" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="43"/>
-      <c r="D28" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E28" s="23"/>
-      <c r="F28" s="44" t="s">
+      <c r="A28" s="52" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="23"/>
+      <c r="D28" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="25"/>
+      <c r="F28" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G28" s="26"/>
+    </row>
+    <row r="29" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="53"/>
+      <c r="B29" s="27">
+        <v>0</v>
+      </c>
+      <c r="C29" s="28"/>
+      <c r="D29" s="27">
+        <v>3</v>
+      </c>
+      <c r="E29" s="28"/>
+      <c r="F29" s="29">
         <v>6</v>
       </c>
-      <c r="G28" s="44"/>
-    </row>
-    <row r="29" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="48"/>
-      <c r="B29" s="26">
-        <v>0</v>
-      </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="26">
+      <c r="G29" s="29"/>
+    </row>
+    <row r="30" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="53" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" s="25"/>
+      <c r="F30" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G30" s="26"/>
+    </row>
+    <row r="31" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="53"/>
+      <c r="B31" s="27">
+        <v>0</v>
+      </c>
+      <c r="C31" s="28"/>
+      <c r="D31" s="27">
         <v>3</v>
       </c>
-      <c r="E29" s="27"/>
-      <c r="F29" s="38">
+      <c r="E31" s="28"/>
+      <c r="F31" s="29">
         <v>6</v>
       </c>
-      <c r="G29" s="38"/>
-    </row>
-    <row r="30" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E30" s="23"/>
-      <c r="F30" s="44" t="s">
+      <c r="G31" s="29"/>
+    </row>
+    <row r="32" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="23"/>
+      <c r="D32" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" s="25"/>
+      <c r="F32" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" s="26"/>
+    </row>
+    <row r="33" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="53"/>
+      <c r="B33" s="41">
+        <v>0</v>
+      </c>
+      <c r="C33" s="42"/>
+      <c r="D33" s="41">
+        <v>3</v>
+      </c>
+      <c r="E33" s="42"/>
+      <c r="F33" s="47">
         <v>6</v>
       </c>
-      <c r="G30" s="44"/>
-    </row>
-    <row r="31" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="48"/>
-      <c r="B31" s="26">
-        <v>0</v>
-      </c>
-      <c r="C31" s="27"/>
-      <c r="D31" s="26">
-        <v>3</v>
-      </c>
-      <c r="E31" s="27"/>
-      <c r="F31" s="38">
-        <v>6</v>
-      </c>
-      <c r="G31" s="38"/>
-    </row>
-    <row r="32" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="43"/>
-      <c r="D32" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E32" s="23"/>
-      <c r="F32" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G32" s="44"/>
-    </row>
-    <row r="33" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="48"/>
-      <c r="B33" s="45">
-        <v>0</v>
-      </c>
-      <c r="C33" s="46"/>
-      <c r="D33" s="45">
-        <v>3</v>
-      </c>
-      <c r="E33" s="46"/>
-      <c r="F33" s="40">
-        <v>6</v>
-      </c>
-      <c r="G33" s="40"/>
+      <c r="G33" s="47"/>
     </row>
     <row r="34" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="42" t="s">
+      <c r="A34" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="23"/>
+      <c r="D34" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="25"/>
+      <c r="F34" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C34" s="43"/>
-      <c r="D34" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" s="23"/>
-      <c r="F34" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="G34" s="44"/>
+      <c r="G34" s="26"/>
     </row>
     <row r="35" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="28"/>
-      <c r="B35" s="45">
-        <v>0</v>
-      </c>
-      <c r="C35" s="46"/>
-      <c r="D35" s="45">
+      <c r="A35" s="43"/>
+      <c r="B35" s="41">
+        <v>0</v>
+      </c>
+      <c r="C35" s="42"/>
+      <c r="D35" s="41">
         <v>2</v>
       </c>
-      <c r="E35" s="46"/>
-      <c r="F35" s="40">
+      <c r="E35" s="42"/>
+      <c r="F35" s="47">
         <v>4</v>
       </c>
-      <c r="G35" s="40"/>
+      <c r="G35" s="47"/>
     </row>
     <row r="36" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="B36" s="32" t="s">
+      <c r="A36" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="C36" s="32" t="s">
+      <c r="D36" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="E36" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="32" t="s">
+      <c r="F36" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="F36" s="32" t="s">
+      <c r="G36" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="G36" s="32" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="37" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="40"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
+      <c r="A37" s="47"/>
+      <c r="B37" s="58"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
     </row>
     <row r="38" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="40"/>
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34"/>
+      <c r="A38" s="47"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="59"/>
+      <c r="D38" s="59"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="59"/>
+      <c r="G38" s="59"/>
     </row>
     <row r="39" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="40"/>
+      <c r="A39" s="47"/>
       <c r="B39" s="2">
         <v>0</v>
       </c>
@@ -1827,48 +1821,48 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="B40" s="32" t="s">
+      <c r="A40" s="60" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="C40" s="32" t="s">
+      <c r="D40" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="E40" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="32" t="s">
+      <c r="F40" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="F40" s="32" t="s">
+      <c r="G40" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="G40" s="32" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="41" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="38"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="33"/>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="33"/>
+      <c r="A41" s="29"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
+      <c r="G41" s="58"/>
     </row>
     <row r="42" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="38"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
+      <c r="A42" s="29"/>
+      <c r="B42" s="59"/>
+      <c r="C42" s="59"/>
+      <c r="D42" s="59"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="59"/>
+      <c r="G42" s="59"/>
     </row>
     <row r="43" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="38"/>
+      <c r="A43" s="29"/>
       <c r="B43" s="2">
         <v>0</v>
       </c>
@@ -1889,48 +1883,48 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="B44" s="32" t="s">
+      <c r="A44" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B44" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="C44" s="32" t="s">
+      <c r="D44" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="D44" s="32" t="s">
+      <c r="E44" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="32" t="s">
+      <c r="F44" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="F44" s="32" t="s">
+      <c r="G44" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="G44" s="32" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="40"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="33"/>
-      <c r="D45" s="33"/>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
-      <c r="G45" s="33"/>
+      <c r="A45" s="47"/>
+      <c r="B45" s="58"/>
+      <c r="C45" s="58"/>
+      <c r="D45" s="58"/>
+      <c r="E45" s="58"/>
+      <c r="F45" s="58"/>
+      <c r="G45" s="58"/>
     </row>
     <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="40"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
+      <c r="A46" s="47"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="59"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="59"/>
+      <c r="F46" s="59"/>
+      <c r="G46" s="59"/>
     </row>
     <row r="47" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="40"/>
+      <c r="A47" s="47"/>
       <c r="B47" s="2">
         <v>0</v>
       </c>
@@ -1951,120 +1945,219 @@
       </c>
     </row>
     <row r="48" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="28" t="s">
+      <c r="A48" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B48" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48" s="50"/>
+      <c r="D48" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="E48" s="50"/>
+      <c r="F48" s="51" t="s">
+        <v>5</v>
+      </c>
+      <c r="G48" s="51"/>
+    </row>
+    <row r="49" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="43"/>
+      <c r="B49" s="27">
+        <v>0</v>
+      </c>
+      <c r="C49" s="28"/>
+      <c r="D49" s="27">
+        <v>1</v>
+      </c>
+      <c r="E49" s="28"/>
+      <c r="F49" s="29">
+        <v>3</v>
+      </c>
+      <c r="G49" s="29"/>
+    </row>
+    <row r="50" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B48" s="35" t="s">
+      <c r="B50" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C50" s="25"/>
+      <c r="D50" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E50" s="25"/>
+      <c r="F50" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="C48" s="36"/>
-      <c r="D48" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="E48" s="36"/>
-      <c r="F48" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="G48" s="37"/>
-    </row>
-    <row r="49" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="28"/>
-      <c r="B49" s="26">
-        <v>0</v>
-      </c>
-      <c r="C49" s="27"/>
-      <c r="D49" s="26">
+      <c r="G50" s="32"/>
+    </row>
+    <row r="51" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="61"/>
+      <c r="B51" s="33">
+        <v>0</v>
+      </c>
+      <c r="C51" s="34"/>
+      <c r="D51" s="33">
         <v>1</v>
       </c>
-      <c r="E49" s="27"/>
-      <c r="F49" s="38">
+      <c r="E51" s="34"/>
+      <c r="F51" s="35">
         <v>3</v>
       </c>
-      <c r="G49" s="38"/>
-    </row>
-    <row r="50" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B50" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C50" s="23"/>
-      <c r="D50" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E50" s="23"/>
-      <c r="F50" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="G50" s="30"/>
-    </row>
-    <row r="51" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="29"/>
-      <c r="B51" s="24">
-        <v>0</v>
-      </c>
-      <c r="C51" s="25"/>
-      <c r="D51" s="24">
-        <v>1</v>
-      </c>
-      <c r="E51" s="25"/>
-      <c r="F51" s="31">
-        <v>3</v>
-      </c>
-      <c r="G51" s="31"/>
+      <c r="G51" s="35"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B52" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C52" s="23"/>
-      <c r="D52" s="42" t="s">
-        <v>101</v>
-      </c>
-      <c r="E52" s="43"/>
-      <c r="F52" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B52" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="G52" s="30"/>
+      <c r="C52" s="25"/>
+      <c r="D52" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="E52" s="23"/>
+      <c r="F52" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="G52" s="32"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B53" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B53" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C53" s="25"/>
-      <c r="D53" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="E53" s="25"/>
-      <c r="F53" s="31" t="s">
+      <c r="C53" s="34"/>
+      <c r="D53" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="E53" s="34"/>
+      <c r="F53" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="G53" s="31"/>
+      <c r="G53" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="153">
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="G44:G46"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="A44:A47"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="D44:D46"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="F44:F46"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="E40:E42"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="G40:G42"/>
+    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="D19:E20"/>
+    <mergeCell ref="F19:G20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="D52:E52"/>
     <mergeCell ref="F52:G52"/>
@@ -2089,120 +2182,21 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="D19:E20"/>
-    <mergeCell ref="F19:G20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="D40:D42"/>
-    <mergeCell ref="E40:E42"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="G40:G42"/>
-    <mergeCell ref="A36:A39"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="G44:G46"/>
-    <mergeCell ref="A48:A49"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="A44:A47"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="D44:D46"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="F44:F46"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -2239,24 +2233,24 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="33" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="D2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>51</v>
-      </c>
     </row>
     <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
+      <c r="A3" s="43"/>
       <c r="B3" s="13">
         <v>0</v>
       </c>
@@ -2271,24 +2265,24 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="33" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>51</v>
-      </c>
     </row>
     <row r="5" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
+      <c r="A5" s="43"/>
       <c r="B5" s="13">
         <v>0</v>
       </c>
@@ -2303,24 +2297,24 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>56</v>
-      </c>
     </row>
     <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="28"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="13">
         <v>0</v>
       </c>
@@ -2335,24 +2329,24 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
-        <v>57</v>
+      <c r="A8" s="46" t="s">
+        <v>55</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="D8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="9" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="28"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="13">
         <v>0</v>
       </c>
@@ -2367,24 +2361,24 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="41" t="s">
-        <v>58</v>
+      <c r="A10" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="E10" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>67</v>
-      </c>
     </row>
     <row r="11" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
+      <c r="A11" s="43"/>
       <c r="B11" s="13">
         <v>0</v>
       </c>
@@ -2399,24 +2393,24 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="E12" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="13" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
+      <c r="A13" s="43"/>
       <c r="B13" s="16">
         <v>0</v>
       </c>
@@ -2432,24 +2426,24 @@
     </row>
     <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="E14" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>1</v>
@@ -2504,19 +2498,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="19" t="s">
         <v>79</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2536,19 +2530,19 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="62" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>83</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2568,19 +2562,19 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2600,19 +2594,19 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="62" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="18" t="s">
-        <v>16</v>
-      </c>
       <c r="E8" s="19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2632,19 +2626,19 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>16</v>
-      </c>
       <c r="E10" s="19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2664,19 +2658,19 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="62" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="18" t="s">
-        <v>16</v>
-      </c>
       <c r="E12" s="19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2696,24 +2690,24 @@
     </row>
     <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="E14" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>1</v>

</xml_diff>